<commit_message>
simply the compute effect size codes + prisma work
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\32283\OneDrive\바탕 화면\meta-analysis\meta-analysis-project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41968A88-5B3A-414A-BA64-97E03FA8C117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061C58E5-4324-47A7-AB18-015CEE7C4F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="549">
   <si>
     <t>Study_ID</t>
   </si>
@@ -748,9 +748,6 @@
   </si>
   <si>
     <t>K-SADS composite</t>
-  </si>
-  <si>
-    <t>raw (imputed)</t>
   </si>
   <si>
     <t>K-SADS 16-item composite (study-specific 4-point averaged scale); MI imputed means (20 datasets, Rubin's rules); N reported = randomized N per Table 1 note.</t>
@@ -1352,14 +1349,6 @@
   </si>
   <si>
     <t>CI_upper_ctrl</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>reported_d_exp</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>reported_d_ctrl</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
@@ -2091,6 +2080,22 @@
   </si>
   <si>
     <t xml:space="preserve">  - With follow-up data                             </t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">raw </t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>raw</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>change_mean_exp</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>change_mean_ctrl</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -2611,16 +2616,16 @@
         <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>17</v>
@@ -2629,10 +2634,10 @@
         <v>18</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>19</v>
@@ -2676,7 +2681,7 @@
         <v>15.63</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>28</v>
@@ -2706,7 +2711,7 @@
         <v>36</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="AA2" s="2" t="s">
         <v>37</v>
@@ -2747,7 +2752,7 @@
         <v>15.6</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>44</v>
@@ -2765,7 +2770,7 @@
         <v>48</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>49</v>
@@ -2777,7 +2782,7 @@
         <v>50</v>
       </c>
       <c r="Z3" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="AA3" s="2" t="s">
         <v>37</v>
@@ -2786,7 +2791,7 @@
         <v>51</v>
       </c>
       <c r="AC3" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="40.799999999999997" customHeight="1">
@@ -2815,10 +2820,10 @@
         <v>55</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>56</v>
@@ -2857,7 +2862,7 @@
         <v>65</v>
       </c>
       <c r="AC4" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="61.2" customHeight="1">
@@ -2889,7 +2894,7 @@
         <v>14.9</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>69</v>
@@ -2925,7 +2930,7 @@
         <v>74</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="AC5" s="2" t="s">
         <v>75</v>
@@ -2960,7 +2965,7 @@
         <v>14.63</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>44</v>
@@ -3342,7 +3347,7 @@
         <v>63</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="AA11" s="2" t="s">
         <v>37</v>
@@ -3365,7 +3370,7 @@
         <v>2018</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>137</v>
@@ -3380,7 +3385,7 @@
         <v>138</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="J12" s="2">
         <v>58.6</v>
@@ -3436,7 +3441,7 @@
         <v>2015</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>147</v>
@@ -3451,10 +3456,10 @@
         <v>26</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>44</v>
@@ -3472,7 +3477,7 @@
         <v>60</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>151</v>
@@ -3484,7 +3489,7 @@
         <v>63</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="AA13" s="2" t="s">
         <v>37</v>
@@ -3501,7 +3506,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C14" s="2">
         <v>2014</v>
@@ -3555,13 +3560,13 @@
         <v>63</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="AA14" s="2" t="s">
         <v>37</v>
       </c>
       <c r="AB14" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="AC14" s="2" t="s">
         <v>159</v>
@@ -3572,7 +3577,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C15" s="2">
         <v>2020</v>
@@ -3626,7 +3631,7 @@
         <v>63</v>
       </c>
       <c r="Z15" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="AA15" s="2" t="s">
         <v>37</v>
@@ -3652,7 +3657,7 @@
         <v>41</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="F16" s="2">
         <v>128</v>
@@ -3673,7 +3678,7 @@
         <v>169</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>170</v>
@@ -3697,7 +3702,7 @@
         <v>50</v>
       </c>
       <c r="Z16" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="AA16" s="2" t="s">
         <v>37</v>
@@ -3706,7 +3711,7 @@
         <v>173</v>
       </c>
       <c r="AC16" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -3714,16 +3719,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="C17" s="2">
         <v>1998</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="N17" s="10"/>
     </row>
@@ -3831,43 +3836,43 @@
         <v>188</v>
       </c>
       <c r="R1" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>404</v>
-      </c>
       <c r="V1" s="1" t="s">
-        <v>405</v>
+        <v>547</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>406</v>
+        <v>548</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="AC1" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="AD1" s="1" t="s">
         <v>399</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>400</v>
       </c>
       <c r="AE1" s="1" t="s">
         <v>22</v>
@@ -3895,32 +3900,20 @@
       <c r="G2" s="2">
         <v>45.99</v>
       </c>
-      <c r="H2" s="2">
-        <v>10.52</v>
-      </c>
       <c r="I2" s="2">
         <v>45.12</v>
       </c>
-      <c r="J2" s="2">
-        <v>12.2</v>
-      </c>
       <c r="K2" s="2">
         <v>36.090000000000003</v>
       </c>
-      <c r="L2" s="2">
-        <v>18.66</v>
-      </c>
       <c r="M2" s="2">
         <v>38.99</v>
       </c>
-      <c r="N2" s="2">
-        <v>16.899999999999999</v>
-      </c>
       <c r="O2" s="2" t="s">
         <v>30</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>191</v>
@@ -3969,35 +3962,23 @@
       <c r="G3" s="2">
         <v>45.99</v>
       </c>
-      <c r="H3" s="2">
-        <v>10.52</v>
-      </c>
       <c r="I3" s="2">
         <v>45.12</v>
       </c>
-      <c r="J3" s="2">
-        <v>12.2</v>
-      </c>
       <c r="K3" s="2">
         <v>35.21</v>
       </c>
-      <c r="L3" s="2">
-        <v>20.74</v>
-      </c>
       <c r="M3" s="2">
         <v>35.86</v>
       </c>
-      <c r="N3" s="2">
-        <v>19.21</v>
-      </c>
       <c r="O3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="R3" s="2">
         <v>-15.99</v>
@@ -4323,41 +4304,29 @@
       <c r="G9" s="2">
         <v>39.6</v>
       </c>
-      <c r="H9" s="2">
-        <v>9.1999999999999993</v>
-      </c>
       <c r="I9" s="2">
         <v>39.5</v>
       </c>
-      <c r="J9" s="2">
-        <v>8.9</v>
-      </c>
       <c r="K9" s="2">
         <v>24.9</v>
       </c>
-      <c r="L9" s="2">
-        <v>8.7899999999999991</v>
-      </c>
       <c r="M9" s="2">
         <v>38.4</v>
       </c>
-      <c r="N9" s="2">
-        <v>8.8000000000000007</v>
-      </c>
       <c r="O9" s="2" t="s">
         <v>71</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="R9" s="2">
+        <v>-18.600000000000001</v>
+      </c>
+      <c r="S9" s="2">
         <v>-10.7</v>
-      </c>
-      <c r="S9" s="2">
-        <v>-18.600000000000001</v>
       </c>
       <c r="T9" s="2">
         <v>-6.3</v>
@@ -4819,15 +4788,6 @@
       <c r="Q17" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="X17" s="2">
-        <v>-0.56999999999999995</v>
-      </c>
-      <c r="Y17" s="2">
-        <v>-0.12</v>
-      </c>
-      <c r="Z17" s="2">
-        <v>-0.35</v>
-      </c>
       <c r="AE17" s="2" t="s">
         <v>219</v>
       </c>
@@ -4879,19 +4839,19 @@
         <v>123</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="X18" s="2">
-        <v>-0.45</v>
+        <v>-0.56999999999999995</v>
       </c>
       <c r="Y18" s="2">
-        <v>0.05</v>
+        <v>-0.12</v>
       </c>
       <c r="Z18" s="2">
-        <v>-0.2</v>
+        <v>-0.35</v>
       </c>
       <c r="AE18" s="2" t="s">
         <v>222</v>
@@ -4944,10 +4904,19 @@
         <v>123</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
+      </c>
+      <c r="X19" s="2">
+        <v>-0.45</v>
+      </c>
+      <c r="Y19" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="Z19" s="2">
+        <v>-0.2</v>
       </c>
       <c r="AE19" s="2" t="s">
         <v>222</v>
@@ -5221,7 +5190,7 @@
         <v>11.9</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>196</v>
@@ -5274,7 +5243,7 @@
         <v>11</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>196</v>
@@ -5604,13 +5573,13 @@
         <v>234</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>235</v>
+        <v>545</v>
       </c>
       <c r="Q31" s="2" t="s">
         <v>196</v>
       </c>
       <c r="AE31" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="30.6">
@@ -5660,13 +5629,13 @@
         <v>234</v>
       </c>
       <c r="P32" s="2" t="s">
-        <v>235</v>
+        <v>545</v>
       </c>
       <c r="Q32" s="2" t="s">
         <v>196</v>
       </c>
       <c r="AE32" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="30.6">
@@ -5716,13 +5685,13 @@
         <v>234</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>235</v>
+        <v>546</v>
       </c>
       <c r="Q33" s="2" t="s">
         <v>196</v>
       </c>
       <c r="AE33" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="30.6">
@@ -5733,7 +5702,7 @@
         <v>233</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D34" s="2">
         <v>18</v>
@@ -5772,13 +5741,13 @@
         <v>234</v>
       </c>
       <c r="P34" s="2" t="s">
-        <v>235</v>
+        <v>545</v>
       </c>
       <c r="Q34" s="2" t="s">
         <v>196</v>
       </c>
       <c r="AE34" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="35" spans="1:31" ht="30.6">
@@ -5828,13 +5797,13 @@
         <v>234</v>
       </c>
       <c r="P35" s="2" t="s">
-        <v>235</v>
+        <v>546</v>
       </c>
       <c r="Q35" s="2" t="s">
         <v>196</v>
       </c>
       <c r="AE35" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -5869,46 +5838,46 @@
   <sheetData>
     <row r="1" spans="1:14" ht="40.799999999999997" customHeight="1">
       <c r="A1" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>250</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="234.6" customHeight="1">
@@ -5916,43 +5885,43 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="K2" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>259</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="163.19999999999999" customHeight="1">
@@ -5960,43 +5929,43 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="J3" s="5" t="s">
+      <c r="K3" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="K3" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="L3" s="5" t="s">
+      <c r="M3" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>266</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="112.2" customHeight="1">
@@ -6004,43 +5973,43 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="J4" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="J4" s="5" t="s">
+      <c r="K4" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="K4" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="L4" s="5" t="s">
+      <c r="M4" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>274</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="163.19999999999999" customHeight="1">
@@ -6048,43 +6017,43 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="G5" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="H5" s="5" t="s">
+      <c r="I5" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="J5" s="5" t="s">
+      <c r="K5" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="L5" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="K5" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="L5" s="5" t="s">
+      <c r="M5" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>281</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="173.4" customHeight="1">
@@ -6092,43 +6061,43 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="G6" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="H6" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="H6" s="5" t="s">
+      <c r="I6" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="J6" s="5" t="s">
+      <c r="K6" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="L6" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="K6" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="L6" s="5" t="s">
+      <c r="M6" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="N6" s="5" t="s">
         <v>288</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="173.4" customHeight="1">
@@ -6136,43 +6105,43 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="F7" s="5" t="s">
+      <c r="G7" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="J7" s="5" t="s">
+      <c r="K7" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="L7" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="K7" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="L7" s="5" t="s">
+      <c r="M7" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="N7" s="5" t="s">
         <v>295</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="132.6" customHeight="1">
@@ -6180,43 +6149,43 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="F8" s="5" t="s">
+      <c r="G8" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="H8" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="H8" s="5" t="s">
+      <c r="I8" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="J8" s="5" t="s">
+      <c r="K8" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="K8" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="L8" s="5" t="s">
+      <c r="M8" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="N8" s="5" t="s">
         <v>302</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="N8" s="5" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="153" customHeight="1">
@@ -6224,43 +6193,43 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="L9" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="L9" s="2" t="s">
+      <c r="M9" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>309</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="132.6" customHeight="1">
@@ -6268,43 +6237,43 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="L10" s="2" t="s">
+      <c r="M10" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N10" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="102" customHeight="1">
@@ -6312,43 +6281,43 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="L11" s="2" t="s">
+      <c r="M11" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>322</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="163.19999999999999" customHeight="1">
@@ -6356,43 +6325,43 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="H12" s="2" t="s">
+      <c r="I12" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J12" s="2" t="s">
+      <c r="K12" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="L12" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="L12" s="2" t="s">
+      <c r="M12" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>329</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="173.4" customHeight="1">
@@ -6400,43 +6369,43 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="H13" s="2" t="s">
+      <c r="I13" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J13" s="2" t="s">
+      <c r="K13" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="K13" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="L13" s="2" t="s">
+      <c r="M13" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>336</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="91.8" customHeight="1">
@@ -6444,43 +6413,43 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="H14" s="2" t="s">
+      <c r="I14" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J14" s="2" t="s">
+      <c r="K14" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="L14" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="L14" s="2" t="s">
+      <c r="M14" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N14" s="2" t="s">
         <v>343</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="51" customHeight="1">
@@ -6488,43 +6457,43 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="H15" s="2" t="s">
+      <c r="I15" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J15" s="2" t="s">
+      <c r="K15" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="L15" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="L15" s="2" t="s">
+      <c r="M15" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="N15" s="2" t="s">
         <v>350</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="163.19999999999999">
@@ -6532,43 +6501,43 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="H16" s="2" t="s">
+      <c r="I16" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="L16" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="L16" s="2" t="s">
+      <c r="M16" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N16" s="2" t="s">
         <v>356</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>357</v>
       </c>
     </row>
   </sheetData>
@@ -6590,19 +6559,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>239</v>
-      </c>
       <c r="C1" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>358</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>359</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -6610,16 +6579,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -6627,19 +6596,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="E3" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>366</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="13.2">
@@ -6647,16 +6616,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -6664,16 +6633,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -6681,19 +6650,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>510</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>371</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>513</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -6701,16 +6670,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -6718,16 +6687,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -6735,16 +6704,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -6752,16 +6721,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="D10" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>496</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -6769,16 +6738,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -6786,16 +6755,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -6803,16 +6772,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -6820,16 +6789,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>447</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>449</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>450</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>452</v>
-      </c>
       <c r="E14" s="4" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -6837,16 +6806,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -6854,16 +6823,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -6871,16 +6840,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -6888,16 +6857,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>460</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>462</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>463</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>452</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -6905,16 +6874,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>465</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>464</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>468</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>466</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -6922,16 +6891,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -6939,16 +6908,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -6956,16 +6925,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -6973,16 +6942,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="D23" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>478</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -6990,16 +6959,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>482</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>484</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>485</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>486</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -7007,16 +6976,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -7024,16 +6993,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -7041,16 +7010,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="D27" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>496</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -7058,16 +7027,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -7078,114 +7047,114 @@
     </row>
     <row r="31" spans="1:5">
       <c r="D31" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>378</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="D32" s="4" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
     </row>
     <row r="33" spans="4:5">
       <c r="D33" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
     </row>
     <row r="34" spans="4:5">
       <c r="D34" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
     </row>
     <row r="35" spans="4:5">
       <c r="D35" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
     </row>
     <row r="36" spans="4:5">
       <c r="D36" s="4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="37" spans="4:5">
       <c r="D37" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="38" spans="4:5">
       <c r="D38" s="4" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="39" spans="4:5">
       <c r="D39" s="4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="40" spans="4:5">
       <c r="D40" s="4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="41" spans="4:5">
       <c r="D41" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
     </row>
     <row r="42" spans="4:5">
       <c r="D42" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="43" spans="4:5">
       <c r="D43" s="4" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="44" spans="4:5">
       <c r="D44" s="4" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
   </sheetData>
@@ -7205,20 +7174,20 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>388</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B4" s="4">
         <v>2748</v>
@@ -7226,7 +7195,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="B6" s="4">
         <v>785</v>
@@ -7234,7 +7203,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="4" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B7" s="4">
         <v>1963</v>
@@ -7242,7 +7211,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B9" s="4">
         <v>1963</v>
@@ -7250,7 +7219,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="4" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B10" s="4">
         <v>1918</v>
@@ -7258,7 +7227,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="4" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B12" s="4">
         <v>46</v>
@@ -7266,7 +7235,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B13" s="4">
         <v>27</v>
@@ -7274,7 +7243,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="4" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="B14" s="4">
         <v>3</v>
@@ -7282,7 +7251,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="4" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="B15" s="4">
         <v>2</v>
@@ -7290,7 +7259,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="B16" s="4">
         <v>3</v>
@@ -7298,7 +7267,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="4" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="B17" s="4">
         <v>6</v>
@@ -7306,7 +7275,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="4" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="B18" s="4">
         <v>6</v>
@@ -7314,7 +7283,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="4" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="B19" s="4">
         <v>2</v>
@@ -7322,7 +7291,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="4" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="B20" s="4">
         <v>0</v>
@@ -7330,7 +7299,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="B21" s="4">
         <v>1</v>
@@ -7338,7 +7307,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="B22" s="4">
         <v>0</v>
@@ -7346,7 +7315,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="4" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="B23" s="4">
         <v>0</v>
@@ -7354,7 +7323,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="4" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="B24" s="4">
         <v>0</v>
@@ -7362,7 +7331,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="4" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="B25" s="4">
         <v>1</v>
@@ -7370,7 +7339,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="15" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="B26" s="4">
         <v>3</v>
@@ -7378,15 +7347,15 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="4" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="4" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="B29" s="4">
         <v>16</v>
@@ -7394,7 +7363,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="4" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="B30" s="4">
         <v>16</v>

</xml_diff>

<commit_message>
solving zero cell problem in acceptability.R + data correction
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\32283\OneDrive\바탕 화면\meta-analysis\meta-analysis-project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C252A67F-AF9C-492C-9C4C-F04BBB8156BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A266206B-D389-4256-A01E-6CA26DD03858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15084" yWindow="0" windowWidth="15408" windowHeight="18480" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15084" yWindow="0" windowWidth="15408" windowHeight="18480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Study_Info" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="561">
   <si>
     <t>Study_ID</t>
   </si>
@@ -485,9 +485,6 @@
     <t>Double-blind placebo-controlled; control=CPE (computerized psychoeducation, matched for length/format); ANCOVA with LOCF; ES calculated as d=(mean change cCBT − mean change CPE)/√error MS</t>
   </si>
   <si>
-    <t>12-18</t>
-  </si>
-  <si>
     <t>Clinical（CAMHS primary mental health workers）</t>
   </si>
   <si>
@@ -593,9 +590,6 @@
     <t>raw</t>
   </si>
   <si>
-    <t>2008 paper Table T3</t>
-  </si>
-  <si>
     <t>Stice 2010</t>
   </si>
   <si>
@@ -608,9 +602,6 @@
     <t>fu_24mo</t>
   </si>
   <si>
-    <t>2010 paper Table</t>
-  </si>
-  <si>
     <t>Bohr 2023</t>
   </si>
   <si>
@@ -672,9 +663,6 @@
   </si>
   <si>
     <t>Stasiak 2014</t>
-  </si>
-  <si>
-    <t>fu_1mo</t>
   </si>
   <si>
     <t>Wright 2020</t>
@@ -2142,10 +2130,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Rohde 2014</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Participants and intervention providers necessarily unblinded due to nature of conditions (book vs. brochure vs. group); three conditions differed significantly on perceived credibility, expected benefit, and satisfaction (all p &lt; .001); however, ITT analysis using multiple imputation (20 datasets, fully conditional specification) was applied for continuous outcomes, and rates of adjunctive mental health treatment did not differ across conditions during follow-up.</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -2228,15 +2212,31 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>2008 paper Table; N=completers; principle: using the first report if later report was different from the former</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Makarushka 2011</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Makarushka, 2011</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>12-18</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>12-16</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2010 paper Table</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rohde 2015</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>fu_1mo</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -2715,7 +2715,7 @@
   <sheetData>
     <row r="1" spans="1:29" ht="51">
       <c r="A1" s="1" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2766,16 +2766,16 @@
         <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>17</v>
@@ -2784,10 +2784,10 @@
         <v>18</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>19</v>
@@ -2846,7 +2846,7 @@
         <v>31</v>
       </c>
       <c r="O2" s="16" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>32</v>
@@ -2861,7 +2861,7 @@
         <v>35</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="AA2" s="2" t="s">
         <v>36</v>
@@ -2881,7 +2881,7 @@
         <v>39</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>558</v>
+        <v>553</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>40</v>
@@ -2902,7 +2902,7 @@
         <v>15.6</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>43</v>
@@ -2917,10 +2917,10 @@
         <v>46</v>
       </c>
       <c r="O3" s="16" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>47</v>
@@ -2932,7 +2932,7 @@
         <v>48</v>
       </c>
       <c r="Z3" s="2" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="AA3" s="2" t="s">
         <v>36</v>
@@ -2941,7 +2941,7 @@
         <v>49</v>
       </c>
       <c r="AC3" s="2" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="40.799999999999997" customHeight="1">
@@ -2970,10 +2970,10 @@
         <v>53</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>54</v>
@@ -2988,7 +2988,7 @@
         <v>57</v>
       </c>
       <c r="O4" s="16" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>58</v>
@@ -3012,7 +3012,7 @@
         <v>62</v>
       </c>
       <c r="AC4" s="2" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="61.2" customHeight="1">
@@ -3044,7 +3044,7 @@
         <v>14.9</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>66</v>
@@ -3059,7 +3059,7 @@
         <v>69</v>
       </c>
       <c r="O5" s="16" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>58</v>
@@ -3077,10 +3077,10 @@
         <v>61</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="AC5" s="2" t="s">
         <v>72</v>
@@ -3272,7 +3272,7 @@
         <v>105</v>
       </c>
       <c r="O8" s="16" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="P8" s="2" t="s">
         <v>94</v>
@@ -3411,7 +3411,7 @@
         <v>69</v>
       </c>
       <c r="O10" s="16" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>32</v>
@@ -3426,7 +3426,7 @@
         <v>60</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="AA10" s="2" t="s">
         <v>36</v>
@@ -3449,7 +3449,7 @@
         <v>2018</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>125</v>
@@ -3464,7 +3464,7 @@
         <v>126</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="J11" s="2">
         <v>58.6</v>
@@ -3482,7 +3482,7 @@
         <v>92</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>94</v>
@@ -3497,7 +3497,7 @@
         <v>130</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="AA11" s="2" t="s">
         <v>36</v>
@@ -3520,7 +3520,7 @@
         <v>2015</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>134</v>
@@ -3532,13 +3532,13 @@
         <v>57</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>26</v>
+        <v>557</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>43</v>
@@ -3553,10 +3553,10 @@
         <v>137</v>
       </c>
       <c r="O12" s="16" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>138</v>
@@ -3568,7 +3568,7 @@
         <v>60</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="AA12" s="2" t="s">
         <v>36</v>
@@ -3585,7 +3585,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="C13" s="2">
         <v>2014</v>
@@ -3642,13 +3642,13 @@
         <v>60</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="AA13" s="2" t="s">
         <v>36</v>
       </c>
       <c r="AB13" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="AC13" s="2" t="s">
         <v>146</v>
@@ -3659,7 +3659,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="C14" s="2">
         <v>2020</v>
@@ -3677,7 +3677,7 @@
         <v>69</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>147</v>
+        <v>556</v>
       </c>
       <c r="I14" s="2">
         <v>15</v>
@@ -3686,10 +3686,10 @@
         <v>64</v>
       </c>
       <c r="K14" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="L14" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>30</v>
@@ -3698,13 +3698,13 @@
         <v>137</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>32</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="R14" s="2">
         <v>45</v>
@@ -3719,16 +3719,16 @@
         <v>60</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="AA14" s="2" t="s">
         <v>36</v>
       </c>
       <c r="AB14" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="AC14" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="AC14" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="204">
@@ -3736,7 +3736,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C15" s="2">
         <v>2015</v>
@@ -3745,7 +3745,7 @@
         <v>40</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="F15" s="2">
         <v>128</v>
@@ -3754,7 +3754,7 @@
         <v>124</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I15" s="2">
         <v>15.5</v>
@@ -3763,16 +3763,16 @@
         <v>68</v>
       </c>
       <c r="K15" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="L15" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="M15" s="2" t="s">
+      <c r="N15" s="10" t="s">
         <v>156</v>
-      </c>
-      <c r="N15" s="10" t="s">
-        <v>157</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>93</v>
@@ -3781,10 +3781,10 @@
         <v>58</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="V15" s="2" t="s">
         <v>34</v>
@@ -3793,19 +3793,19 @@
         <v>48</v>
       </c>
       <c r="X15" s="2" t="s">
-        <v>554</v>
+        <v>549</v>
       </c>
       <c r="Z15" s="2" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="AA15" s="2" t="s">
         <v>36</v>
       </c>
       <c r="AB15" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AC15" s="2" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="142.80000000000001">
@@ -3813,16 +3813,16 @@
         <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="C16" s="2">
         <v>1998</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="F16" s="2">
         <v>15</v>
@@ -3831,7 +3831,7 @@
         <v>15</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="I16" s="2">
         <v>15.89</v>
@@ -3840,52 +3840,52 @@
         <v>63.6</v>
       </c>
       <c r="K16" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>508</v>
+      </c>
+      <c r="O16" s="16" t="s">
+        <v>509</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="R16" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="L16" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="N16" s="10" t="s">
+      <c r="V16" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="O16" s="16" t="s">
+      <c r="W16" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="X16" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="Y16" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="Z16" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="AA16" s="2" t="s">
         <v>514</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="R16" s="2" t="s">
-        <v>551</v>
-      </c>
-      <c r="V16" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="W16" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="X16" s="2" t="s">
-        <v>554</v>
-      </c>
-      <c r="Y16" s="2" t="s">
-        <v>550</v>
-      </c>
-      <c r="Z16" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="AA16" s="2" t="s">
-        <v>518</v>
-      </c>
       <c r="AB16" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="AC16" s="2" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
     </row>
     <row r="17" spans="14:14">
@@ -3947,88 +3947,88 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="Q1" s="1" t="s">
-        <v>174</v>
-      </c>
       <c r="R1" s="1" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="U1" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="V1" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>370</v>
-      </c>
       <c r="AA1" s="1" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="AB1" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="AD1" s="1" t="s">
         <v>358</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>362</v>
       </c>
       <c r="AE1" s="1" t="s">
         <v>22</v>
@@ -4039,10 +4039,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="D2" s="2">
         <v>3</v>
@@ -4069,10 +4069,10 @@
         <v>30</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="R2" s="2">
         <v>-14.34</v>
@@ -4093,13 +4093,13 @@
         <v>-6.13</v>
       </c>
       <c r="AC2" s="2">
+        <v>17</v>
+      </c>
+      <c r="AD2" s="2">
         <v>15</v>
       </c>
-      <c r="AD2" s="2">
-        <v>17</v>
-      </c>
       <c r="AE2" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:31">
@@ -4107,19 +4107,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D3" s="2">
         <v>6</v>
       </c>
       <c r="E3" s="2">
+        <v>61</v>
+      </c>
+      <c r="F3" s="2">
         <v>68</v>
-      </c>
-      <c r="F3" s="2">
-        <v>70</v>
       </c>
       <c r="G3" s="2">
         <v>45.99</v>
@@ -4137,10 +4137,10 @@
         <v>30</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="R3" s="2">
         <v>-15.99</v>
@@ -4161,27 +4161,27 @@
         <v>-9.26</v>
       </c>
       <c r="AE3" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="4" spans="1:31" ht="20.399999999999999">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31">
       <c r="A4" s="2">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
       </c>
       <c r="E4" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F4" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G4" s="2">
         <v>18.2</v>
@@ -4211,10 +4211,10 @@
         <v>45</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC4" s="2">
         <v>4</v>
@@ -4223,7 +4223,7 @@
         <v>1</v>
       </c>
       <c r="AE4" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="5" spans="1:31">
@@ -4231,19 +4231,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D5" s="2">
         <v>6</v>
       </c>
       <c r="E5" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F5" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G5" s="2">
         <v>18.2</v>
@@ -4273,13 +4273,13 @@
         <v>45</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE5" s="2" t="s">
-        <v>183</v>
+        <v>558</v>
       </c>
     </row>
     <row r="6" spans="1:31">
@@ -4287,19 +4287,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D6" s="2">
         <v>12</v>
       </c>
       <c r="E6" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F6" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G6" s="2">
         <v>18.2</v>
@@ -4329,13 +4329,13 @@
         <v>45</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE6" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:31">
@@ -4343,19 +4343,19 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D7" s="2">
         <v>24</v>
       </c>
       <c r="E7" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F7" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G7" s="2">
         <v>18.2</v>
@@ -4385,13 +4385,13 @@
         <v>45</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE7" s="2" t="s">
-        <v>188</v>
+        <v>558</v>
       </c>
     </row>
     <row r="8" spans="1:31" ht="20.399999999999999" customHeight="1">
@@ -4399,10 +4399,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D8" s="2">
         <v>2</v>
@@ -4414,10 +4414,10 @@
         <v>19</v>
       </c>
       <c r="G8" s="2">
-        <v>21.2</v>
+        <v>22.9</v>
       </c>
       <c r="H8" s="2">
-        <v>7.6</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="I8" s="2">
         <v>25.5</v>
@@ -4426,25 +4426,25 @@
         <v>8.5399999999999991</v>
       </c>
       <c r="K8" s="2">
+        <v>23.21</v>
+      </c>
+      <c r="L8" s="2">
+        <v>8.86</v>
+      </c>
+      <c r="M8" s="2">
         <v>23.68</v>
       </c>
-      <c r="L8" s="2">
+      <c r="N8" s="2">
         <v>8.58</v>
-      </c>
-      <c r="M8" s="2">
-        <v>23.21</v>
-      </c>
-      <c r="N8" s="2">
-        <v>8.86</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>56</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC8" s="2">
         <v>7</v>
@@ -4453,7 +4453,7 @@
         <v>9</v>
       </c>
       <c r="AE8" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:31">
@@ -4461,10 +4461,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D9" s="2">
         <v>1.5</v>
@@ -4491,10 +4491,10 @@
         <v>68</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="R9" s="2">
         <v>-18.600000000000001</v>
@@ -4521,7 +4521,7 @@
         <v>0</v>
       </c>
       <c r="AE9" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:31">
@@ -4529,10 +4529,10 @@
         <v>5</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D10" s="2">
         <v>8</v>
@@ -4571,10 +4571,10 @@
         <v>56</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC10" s="2">
         <v>7</v>
@@ -4583,7 +4583,7 @@
         <v>0</v>
       </c>
       <c r="AE10" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="11" spans="1:31">
@@ -4591,10 +4591,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D11" s="2">
         <v>12</v>
@@ -4633,13 +4633,13 @@
         <v>56</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE11" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:31">
@@ -4647,10 +4647,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D12" s="2">
         <v>1.5</v>
@@ -4689,19 +4689,19 @@
         <v>91</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC12" s="2">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="AD12" s="2">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="AE12" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" spans="1:31">
@@ -4709,10 +4709,10 @@
         <v>6</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D13" s="2">
         <v>6</v>
@@ -4751,13 +4751,13 @@
         <v>91</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE13" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="1:31" ht="30.6" customHeight="1">
@@ -4765,10 +4765,10 @@
         <v>8</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D14" s="2">
         <v>1</v>
@@ -4807,10 +4807,10 @@
         <v>112</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC14" s="2">
         <v>17</v>
@@ -4819,7 +4819,7 @@
         <v>13</v>
       </c>
       <c r="AE14" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="15" spans="1:31" ht="30.6" customHeight="1">
@@ -4827,10 +4827,10 @@
         <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D15" s="2">
         <v>3</v>
@@ -4869,13 +4869,13 @@
         <v>112</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE15" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:31" ht="30.6" customHeight="1">
@@ -4883,13 +4883,13 @@
         <v>9</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D16" s="2">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="E16" s="2">
         <v>130</v>
@@ -4925,10 +4925,10 @@
         <v>112</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="X16" s="2">
         <v>-0.56999999999999995</v>
@@ -4946,7 +4946,7 @@
         <v>36</v>
       </c>
       <c r="AE16" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="30.6" customHeight="1">
@@ -4954,10 +4954,10 @@
         <v>9</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D17" s="2">
         <v>4</v>
@@ -4996,10 +4996,10 @@
         <v>112</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="X17" s="2">
         <v>-0.45</v>
@@ -5011,7 +5011,7 @@
         <v>-0.2</v>
       </c>
       <c r="AE17" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:31">
@@ -5019,10 +5019,10 @@
         <v>10</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D18" s="2">
         <v>0</v>
@@ -5058,13 +5058,13 @@
         <v>12.56</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC18" s="2">
         <v>2</v>
@@ -5073,7 +5073,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="19" spans="1:31">
@@ -5081,10 +5081,10 @@
         <v>10</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D19" s="2">
         <v>3</v>
@@ -5120,16 +5120,16 @@
         <v>13.04</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE19" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:31">
@@ -5137,10 +5137,10 @@
         <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D20" s="2">
         <v>6</v>
@@ -5176,16 +5176,16 @@
         <v>13.33</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE20" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:31">
@@ -5193,10 +5193,10 @@
         <v>10</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D21" s="2">
         <v>12</v>
@@ -5232,16 +5232,16 @@
         <v>15.03</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="P21" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE21" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:31">
@@ -5249,10 +5249,10 @@
         <v>11</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D22" s="2">
         <v>2</v>
@@ -5288,13 +5288,13 @@
         <v>11.9</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC22" s="2">
         <v>3</v>
@@ -5308,10 +5308,10 @@
         <v>11</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D23" s="2">
         <v>4</v>
@@ -5347,13 +5347,13 @@
         <v>11</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="61.2" customHeight="1">
@@ -5361,10 +5361,10 @@
         <v>12</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D24" s="2">
         <v>2</v>
@@ -5403,10 +5403,10 @@
         <v>136</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q24" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC24" s="2">
         <v>0</v>
@@ -5423,19 +5423,19 @@
         <v>13</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D25" s="2">
         <v>1.5</v>
       </c>
       <c r="E25" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F25" s="2">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G25" s="2">
         <v>48.29</v>
@@ -5465,10 +5465,10 @@
         <v>68</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC25" s="2">
         <v>1</v>
@@ -5482,19 +5482,19 @@
         <v>13</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>210</v>
+        <v>560</v>
       </c>
       <c r="D26" s="2">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E26" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F26" s="2">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G26" s="2">
         <v>48.29</v>
@@ -5524,10 +5524,10 @@
         <v>68</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" spans="1:31" ht="132.6" customHeight="1">
@@ -5535,10 +5535,10 @@
         <v>14</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D27" s="2">
         <v>4</v>
@@ -5577,10 +5577,10 @@
         <v>45</v>
       </c>
       <c r="P27" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q27" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC27" s="2">
         <v>28</v>
@@ -5589,7 +5589,7 @@
         <v>25</v>
       </c>
       <c r="AE27" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="28" spans="1:31" ht="132.6" customHeight="1">
@@ -5597,10 +5597,10 @@
         <v>14</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D28" s="2">
         <v>12</v>
@@ -5639,13 +5639,13 @@
         <v>45</v>
       </c>
       <c r="P28" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q28" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE28" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:31" ht="30.6">
@@ -5653,19 +5653,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D29" s="2">
         <v>2</v>
       </c>
       <c r="E29" s="2">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="F29" s="2">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="G29" s="2">
         <v>1.45</v>
@@ -5692,13 +5692,13 @@
         <v>0.41</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="P29" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="Q29" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC29" s="2">
         <v>6</v>
@@ -5707,7 +5707,7 @@
         <v>8</v>
       </c>
       <c r="AE29" s="2" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="30.6">
@@ -5715,19 +5715,19 @@
         <v>15</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D30" s="2">
         <v>6</v>
       </c>
       <c r="E30" s="2">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="F30" s="2">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="G30" s="2">
         <v>1.45</v>
@@ -5754,16 +5754,16 @@
         <v>0.33</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="P30" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE30" s="2" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="31" spans="1:31" ht="30.6">
@@ -5771,19 +5771,19 @@
         <v>15</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D31" s="2">
         <v>12</v>
       </c>
       <c r="E31" s="2">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F31" s="2">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="G31" s="2">
         <v>1.45</v>
@@ -5810,16 +5810,16 @@
         <v>0.4</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE31" s="2" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="30.6">
@@ -5827,19 +5827,19 @@
         <v>15</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D32" s="2">
         <v>18</v>
       </c>
       <c r="E32" s="2">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="F32" s="2">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="G32" s="2">
         <v>1.45</v>
@@ -5866,16 +5866,16 @@
         <v>0.35</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="P32" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="Q32" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE32" s="2" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="30.6">
@@ -5883,19 +5883,19 @@
         <v>15</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D33" s="2">
         <v>24</v>
       </c>
       <c r="E33" s="2">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="F33" s="2">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="G33" s="2">
         <v>1.45</v>
@@ -5922,16 +5922,16 @@
         <v>0.43</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="Q33" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE33" s="2" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="51">
@@ -5939,10 +5939,10 @@
         <v>16</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="D34" s="2">
         <v>1</v>
@@ -5978,13 +5978,13 @@
         <v>5.2</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="P34" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="Q34" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="AC34" s="2">
         <v>3</v>
@@ -5993,7 +5993,7 @@
         <v>5</v>
       </c>
       <c r="AE34" s="2" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
     </row>
   </sheetData>
@@ -6028,46 +6028,46 @@
   <sheetData>
     <row r="1" spans="1:14" ht="40.799999999999997" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>226</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="234.6" customHeight="1">
@@ -6075,43 +6075,43 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="I2" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="K2" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="M2" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>234</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="163.19999999999999" customHeight="1">
@@ -6119,43 +6119,43 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="K3" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="M3" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="112.2" customHeight="1">
@@ -6163,43 +6163,43 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="I4" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="J4" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="K4" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="M4" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>249</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="163.19999999999999" customHeight="1">
@@ -6207,43 +6207,43 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="K5" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="L5" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="M5" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>256</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="173.4" customHeight="1">
@@ -6251,43 +6251,43 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="K6" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="L6" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="M6" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="N6" s="5" t="s">
         <v>263</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="173.4" customHeight="1">
@@ -6295,43 +6295,43 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="L7" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>272</v>
-      </c>
       <c r="M7" s="5" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="153" customHeight="1">
@@ -6339,43 +6339,43 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="K8" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="M8" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="132.6" customHeight="1">
@@ -6383,43 +6383,43 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="K9" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="L9" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="M9" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>283</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="102" customHeight="1">
@@ -6427,43 +6427,43 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="M10" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N10" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="163.19999999999999" customHeight="1">
@@ -6471,43 +6471,43 @@
         <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>537</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>298</v>
-      </c>
       <c r="M11" s="2" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="173.4" customHeight="1">
@@ -6515,43 +6515,43 @@
         <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="K12" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="L12" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="M12" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>301</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="91.8" customHeight="1">
@@ -6559,43 +6559,43 @@
         <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="M13" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="51" customHeight="1">
@@ -6603,43 +6603,43 @@
         <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="N14" s="2" t="s">
         <v>312</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>556</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="204">
@@ -6647,43 +6647,43 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N15" s="2" t="s">
         <v>317</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>553</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="91.8">
@@ -6691,43 +6691,43 @@
         <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="K16" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="L16" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="M16" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="N16" s="2" t="s">
         <v>523</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>526</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>527</v>
       </c>
     </row>
   </sheetData>
@@ -6750,19 +6750,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -6770,16 +6770,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -6787,19 +6787,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="13.2">
@@ -6807,16 +6807,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -6824,16 +6824,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -6841,19 +6841,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -6861,16 +6861,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -6878,16 +6878,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -6895,16 +6895,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -6912,16 +6912,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -6929,16 +6929,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -6946,16 +6946,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -6963,16 +6963,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -6980,16 +6980,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -6997,16 +6997,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -7014,16 +7014,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -7031,16 +7031,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -7048,16 +7048,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -7065,16 +7065,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>422</v>
       </c>
-      <c r="C19" s="14" t="s">
-        <v>426</v>
-      </c>
       <c r="D19" s="4" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -7082,16 +7082,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -7099,16 +7099,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -7116,16 +7116,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -7133,16 +7133,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -7150,16 +7150,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -7167,16 +7167,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -7184,16 +7184,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -7201,16 +7201,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="C27" s="14" t="s">
+        <v>449</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>453</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>454</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -7218,16 +7218,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="30.6">
@@ -7235,19 +7235,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>535</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>538</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>539</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>476</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>540</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -7255,114 +7255,114 @@
     </row>
     <row r="31" spans="1:6">
       <c r="D31" s="4" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="D32" s="4" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="33" spans="4:5">
       <c r="D33" s="4" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
     </row>
     <row r="34" spans="4:5">
       <c r="D34" s="4" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="35" spans="4:5">
       <c r="D35" s="4" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
     </row>
     <row r="36" spans="4:5">
       <c r="D36" s="4" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
     <row r="37" spans="4:5">
       <c r="D37" s="4" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="38" spans="4:5">
       <c r="D38" s="4" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
     </row>
     <row r="39" spans="4:5">
       <c r="D39" s="4" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
     </row>
     <row r="40" spans="4:5">
       <c r="D40" s="4" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="41" spans="4:5">
       <c r="D41" s="4" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="42" spans="4:5">
       <c r="D42" s="4" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="43" spans="4:5">
       <c r="D43" s="4" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
     </row>
     <row r="44" spans="4:5">
       <c r="D44" s="4" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -7382,20 +7382,20 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="4" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="4" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="4" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="B4" s="4">
         <v>2748</v>
@@ -7403,7 +7403,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="B6" s="4">
         <v>785</v>
@@ -7411,7 +7411,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="4" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="B7" s="4">
         <v>1963</v>
@@ -7419,7 +7419,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="B9" s="4">
         <v>1963</v>
@@ -7427,7 +7427,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="4" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="B10" s="4">
         <v>1918</v>
@@ -7435,7 +7435,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="4" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="B12" s="4">
         <v>46</v>
@@ -7443,7 +7443,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="4" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="B13" s="4">
         <v>28</v>
@@ -7451,7 +7451,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="4" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="B14" s="4">
         <v>3</v>
@@ -7459,7 +7459,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="4" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="B15" s="4">
         <v>2</v>
@@ -7467,7 +7467,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="B16" s="4">
         <v>3</v>
@@ -7475,7 +7475,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="4" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="B17" s="4">
         <v>6</v>
@@ -7483,7 +7483,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="4" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="B18" s="4">
         <v>6</v>
@@ -7491,7 +7491,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="4" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="B19" s="4">
         <v>3</v>
@@ -7499,7 +7499,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="4" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="B20" s="4">
         <v>0</v>
@@ -7507,7 +7507,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="B21" s="4">
         <v>1</v>
@@ -7515,7 +7515,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="B22" s="4">
         <v>0</v>
@@ -7523,7 +7523,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="4" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="B23" s="4">
         <v>0</v>
@@ -7531,7 +7531,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="4" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="B24" s="4">
         <v>0</v>
@@ -7539,7 +7539,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="4" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="B25" s="4">
         <v>1</v>
@@ -7547,7 +7547,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="15" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="B26" s="4">
         <v>3</v>
@@ -7555,15 +7555,15 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="4" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="4" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="B29" s="4">
         <v>16</v>
@@ -7571,7 +7571,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="4" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="B30" s="4">
         <v>16</v>

</xml_diff>

<commit_message>
acceptability revised + dropout data correction
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\32283\OneDrive\바탕 화면\meta-analysis\meta-analysis-project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A266206B-D389-4256-A01E-6CA26DD03858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78F498D-1A4A-4409-AA9A-4C8D28E5A9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15084" yWindow="0" windowWidth="15408" windowHeight="18480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4518,7 +4518,7 @@
         <v>1</v>
       </c>
       <c r="AD9" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE9" s="2" t="s">
         <v>189</v>
@@ -5067,7 +5067,7 @@
         <v>181</v>
       </c>
       <c r="AC18" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD18" s="2">
         <v>0</v>

</xml_diff>

<commit_message>
dropouts varies, considering hanlding zero cells might not enough -> clarify the heterogenity source accdording to the advice of PKU stranger, remember her name is moki
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\32283\OneDrive\바탕 화면\meta-analysis\meta-analysis-project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78F498D-1A4A-4409-AA9A-4C8D28E5A9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32FF973B-9DDE-4A44-87FE-CC51E0E44219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15084" yWindow="0" windowWidth="15408" windowHeight="18480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Study_Info" sheetId="1" r:id="rId1"/>

</xml_diff>